<commit_message>
final result was done
</commit_message>
<xml_diff>
--- a/outputs/evaluacion_integral_lora_vs_hiperparametros/evaluacion_integral_lora_vs_hiperparametros.xlsx
+++ b/outputs/evaluacion_integral_lora_vs_hiperparametros/evaluacion_integral_lora_vs_hiperparametros.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1851,7 +1851,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2822,7 +2822,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3373,7 +3373,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3825,7 +3825,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -23925,7 +23925,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -24061,7 +24061,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -24197,7 +24197,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -24333,7 +24333,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -24469,7 +24469,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -24605,7 +24605,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -24741,7 +24741,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -24877,7 +24877,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -25013,7 +25013,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -25149,7 +25149,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -25285,7 +25285,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -25421,7 +25421,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -25557,7 +25557,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -25693,7 +25693,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -25829,7 +25829,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -25965,7 +25965,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -26101,7 +26101,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -26237,7 +26237,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -26373,7 +26373,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -26509,7 +26509,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -26645,7 +26645,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -26781,7 +26781,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -26917,7 +26917,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -27053,7 +27053,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -27189,7 +27189,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -27325,7 +27325,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -27461,7 +27461,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -27733,7 +27733,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -27869,7 +27869,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -28005,7 +28005,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -28141,7 +28141,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -28277,7 +28277,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -28413,7 +28413,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -28549,7 +28549,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -28685,7 +28685,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -28821,7 +28821,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -28957,7 +28957,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -29093,7 +29093,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -29229,7 +29229,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -29365,7 +29365,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -29501,7 +29501,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -29637,7 +29637,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -29773,7 +29773,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -29909,7 +29909,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -30045,7 +30045,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -30317,7 +30317,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -30453,7 +30453,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -30589,7 +30589,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -30725,7 +30725,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -30861,7 +30861,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -30997,7 +30997,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -31133,7 +31133,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -31269,7 +31269,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -31405,7 +31405,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -31541,7 +31541,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -31677,7 +31677,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -31813,7 +31813,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -31949,7 +31949,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -32085,7 +32085,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -32221,7 +32221,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -32357,7 +32357,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -32493,7 +32493,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -32629,7 +32629,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -32765,7 +32765,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -32901,7 +32901,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -33037,7 +33037,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -33173,7 +33173,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -33309,7 +33309,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -33445,7 +33445,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -33581,7 +33581,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -49157,7 +49157,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -49263,7 +49263,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -49369,7 +49369,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -49475,7 +49475,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -49581,7 +49581,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -49687,7 +49687,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -49793,7 +49793,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -49899,7 +49899,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -50005,7 +50005,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -50111,7 +50111,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -50217,7 +50217,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -50323,7 +50323,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -50429,7 +50429,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -50535,7 +50535,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -50641,7 +50641,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -50747,7 +50747,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -50853,7 +50853,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -50959,7 +50959,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -51065,7 +51065,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -51171,7 +51171,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -51277,7 +51277,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -51383,7 +51383,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -51489,7 +51489,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -51595,7 +51595,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -51701,7 +51701,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -51807,7 +51807,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -51913,7 +51913,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -52019,7 +52019,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -52125,7 +52125,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -52231,7 +52231,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -52337,7 +52337,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -52443,7 +52443,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -52549,7 +52549,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -52655,7 +52655,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -52761,7 +52761,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -52867,7 +52867,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -52973,7 +52973,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -53079,7 +53079,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -53185,7 +53185,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -53291,7 +53291,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -53397,7 +53397,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -53503,7 +53503,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -53609,7 +53609,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -53715,7 +53715,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -53821,7 +53821,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -53927,7 +53927,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -54033,7 +54033,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -54139,7 +54139,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -54245,7 +54245,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -54351,7 +54351,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -54457,7 +54457,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -54563,7 +54563,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -54669,7 +54669,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -54775,7 +54775,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -54881,7 +54881,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -54987,7 +54987,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -55093,7 +55093,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -55199,7 +55199,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -55305,7 +55305,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -55411,7 +55411,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -55517,7 +55517,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -55623,7 +55623,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -55729,7 +55729,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -55835,7 +55835,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -55941,7 +55941,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -56047,7 +56047,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -56153,7 +56153,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -56259,7 +56259,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -56365,7 +56365,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -56471,7 +56471,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -56577,7 +56577,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -56683,7 +56683,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -67733,7 +67733,7 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O146" t="n">
@@ -67808,7 +67808,7 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O147" t="n">
@@ -67883,7 +67883,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O148" t="n">
@@ -67958,7 +67958,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O149" t="n">
@@ -68033,7 +68033,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O150" t="n">
@@ -68108,7 +68108,7 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O151" t="n">
@@ -68183,7 +68183,7 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O152" t="n">
@@ -68258,7 +68258,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O153" t="n">
@@ -68333,7 +68333,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O154" t="n">
@@ -68408,7 +68408,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O155" t="n">
@@ -68483,7 +68483,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O156" t="n">
@@ -68558,7 +68558,7 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O157" t="n">
@@ -68633,7 +68633,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O158" t="n">
@@ -68708,7 +68708,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O159" t="n">
@@ -68783,7 +68783,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O160" t="n">
@@ -68858,7 +68858,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O161" t="n">
@@ -68933,7 +68933,7 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O162" t="n">
@@ -69008,7 +69008,7 @@
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O163" t="n">
@@ -69083,7 +69083,7 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O164" t="n">
@@ -69158,7 +69158,7 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O165" t="n">
@@ -69233,7 +69233,7 @@
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O166" t="n">
@@ -69308,7 +69308,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O167" t="n">
@@ -69383,7 +69383,7 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O168" t="n">
@@ -69458,7 +69458,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O169" t="n">
@@ -69533,7 +69533,7 @@
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O170" t="n">
@@ -69608,7 +69608,7 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O171" t="n">
@@ -69683,7 +69683,7 @@
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O172" t="n">
@@ -69758,7 +69758,7 @@
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O173" t="n">
@@ -69833,7 +69833,7 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O174" t="n">
@@ -69908,7 +69908,7 @@
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O175" t="n">
@@ -69983,7 +69983,7 @@
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O176" t="n">
@@ -70058,7 +70058,7 @@
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O177" t="n">
@@ -70133,7 +70133,7 @@
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O178" t="n">
@@ -70208,7 +70208,7 @@
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O179" t="n">
@@ -70283,7 +70283,7 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O180" t="n">
@@ -70358,7 +70358,7 @@
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>lora_llama3</t>
+          <t>lora_mistral</t>
         </is>
       </c>
       <c r="O181" t="n">
@@ -70433,7 +70433,7 @@
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O182" t="n">
@@ -70508,7 +70508,7 @@
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O183" t="n">
@@ -70583,7 +70583,7 @@
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O184" t="n">
@@ -70658,7 +70658,7 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O185" t="n">
@@ -70733,7 +70733,7 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O186" t="n">
@@ -70808,7 +70808,7 @@
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O187" t="n">
@@ -70883,7 +70883,7 @@
       </c>
       <c r="N188" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O188" t="n">
@@ -70958,7 +70958,7 @@
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O189" t="n">
@@ -71033,7 +71033,7 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O190" t="n">
@@ -71108,7 +71108,7 @@
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O191" t="n">
@@ -71183,7 +71183,7 @@
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O192" t="n">
@@ -71258,7 +71258,7 @@
       </c>
       <c r="N193" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O193" t="n">
@@ -71333,7 +71333,7 @@
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O194" t="n">
@@ -71408,7 +71408,7 @@
       </c>
       <c r="N195" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O195" t="n">
@@ -71483,7 +71483,7 @@
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O196" t="n">
@@ -71558,7 +71558,7 @@
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O197" t="n">
@@ -71633,7 +71633,7 @@
       </c>
       <c r="N198" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O198" t="n">
@@ -71708,7 +71708,7 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O199" t="n">
@@ -71783,7 +71783,7 @@
       </c>
       <c r="N200" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O200" t="n">
@@ -71858,7 +71858,7 @@
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O201" t="n">
@@ -71933,7 +71933,7 @@
       </c>
       <c r="N202" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O202" t="n">
@@ -72008,7 +72008,7 @@
       </c>
       <c r="N203" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O203" t="n">
@@ -72083,7 +72083,7 @@
       </c>
       <c r="N204" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O204" t="n">
@@ -72158,7 +72158,7 @@
       </c>
       <c r="N205" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O205" t="n">
@@ -72233,7 +72233,7 @@
       </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O206" t="n">
@@ -72308,7 +72308,7 @@
       </c>
       <c r="N207" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O207" t="n">
@@ -72383,7 +72383,7 @@
       </c>
       <c r="N208" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O208" t="n">
@@ -72458,7 +72458,7 @@
       </c>
       <c r="N209" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O209" t="n">
@@ -72533,7 +72533,7 @@
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O210" t="n">
@@ -72608,7 +72608,7 @@
       </c>
       <c r="N211" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O211" t="n">
@@ -72683,7 +72683,7 @@
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O212" t="n">
@@ -72758,7 +72758,7 @@
       </c>
       <c r="N213" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O213" t="n">
@@ -72833,7 +72833,7 @@
       </c>
       <c r="N214" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O214" t="n">
@@ -72908,7 +72908,7 @@
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O215" t="n">
@@ -72983,7 +72983,7 @@
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O216" t="n">
@@ -73058,7 +73058,7 @@
       </c>
       <c r="N217" t="inlineStr">
         <is>
-          <t>lora_mistral</t>
+          <t>lora_llama3</t>
         </is>
       </c>
       <c r="O217" t="n">

</xml_diff>